<commit_message>
Final push, everything should be good now, added comments removed a file and added it to the test file. Hopefully everything is correct now...
</commit_message>
<xml_diff>
--- a/weights/baseline_results.xlsx
+++ b/weights/baseline_results.xlsx
@@ -1025,367 +1025,367 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>124.5</v>
+        <v>401.7</v>
       </c>
       <c r="B2" t="n">
-        <v>17.70451919708638</v>
+        <v>127.8366535857381</v>
       </c>
       <c r="C2" t="n">
+        <v>215</v>
+      </c>
+      <c r="D2" t="n">
+        <v>510</v>
+      </c>
+      <c r="E2" t="n">
+        <v>349.7</v>
+      </c>
+      <c r="F2" t="n">
+        <v>137.5667474355631</v>
+      </c>
+      <c r="G2" t="n">
+        <v>210</v>
+      </c>
+      <c r="H2" t="n">
+        <v>534</v>
+      </c>
+      <c r="I2" t="n">
+        <v>1580.3</v>
+      </c>
+      <c r="J2" t="n">
+        <v>1513.900528436396</v>
+      </c>
+      <c r="K2" t="n">
+        <v>208</v>
+      </c>
+      <c r="L2" t="n">
+        <v>4005</v>
+      </c>
+      <c r="M2" t="n">
+        <v>1297.7</v>
+      </c>
+      <c r="N2" t="n">
+        <v>1850.305599083568</v>
+      </c>
+      <c r="O2" t="n">
+        <v>191</v>
+      </c>
+      <c r="P2" t="n">
+        <v>6141</v>
+      </c>
+      <c r="Q2" t="n">
+        <v>575.3</v>
+      </c>
+      <c r="R2" t="n">
+        <v>890.1296590946736</v>
+      </c>
+      <c r="S2" t="n">
+        <v>192</v>
+      </c>
+      <c r="T2" t="n">
+        <v>3232</v>
+      </c>
+      <c r="U2" t="n">
+        <v>236.2</v>
+      </c>
+      <c r="V2" t="n">
+        <v>25.49039034616771</v>
+      </c>
+      <c r="W2" t="n">
+        <v>174</v>
+      </c>
+      <c r="X2" t="n">
+        <v>274</v>
+      </c>
+      <c r="Y2" t="n">
+        <v>252.6</v>
+      </c>
+      <c r="Z2" t="n">
+        <v>93.96084290809655</v>
+      </c>
+      <c r="AA2" t="n">
+        <v>168</v>
+      </c>
+      <c r="AB2" t="n">
+        <v>527</v>
+      </c>
+      <c r="AC2" t="n">
+        <v>241.5</v>
+      </c>
+      <c r="AD2" t="n">
+        <v>89.81898463019942</v>
+      </c>
+      <c r="AE2" t="n">
+        <v>177</v>
+      </c>
+      <c r="AF2" t="n">
+        <v>505</v>
+      </c>
+      <c r="AG2" t="n">
+        <v>204.2</v>
+      </c>
+      <c r="AH2" t="n">
+        <v>17.28467529344998</v>
+      </c>
+      <c r="AI2" t="n">
+        <v>173</v>
+      </c>
+      <c r="AJ2" t="n">
+        <v>224</v>
+      </c>
+      <c r="AK2" t="n">
+        <v>170.9</v>
+      </c>
+      <c r="AL2" t="n">
+        <v>17.76203817133608</v>
+      </c>
+      <c r="AM2" t="n">
+        <v>146</v>
+      </c>
+      <c r="AN2" t="n">
+        <v>200</v>
+      </c>
+      <c r="AO2" t="n">
+        <v>174.7</v>
+      </c>
+      <c r="AP2" t="n">
+        <v>25.1716109933393</v>
+      </c>
+      <c r="AQ2" t="n">
+        <v>147</v>
+      </c>
+      <c r="AR2" t="n">
+        <v>218</v>
+      </c>
+      <c r="AS2" t="n">
+        <v>147.9</v>
+      </c>
+      <c r="AT2" t="n">
+        <v>41.30242123653285</v>
+      </c>
+      <c r="AU2" t="n">
+        <v>105</v>
+      </c>
+      <c r="AV2" t="n">
+        <v>216</v>
+      </c>
+      <c r="AW2" t="n">
+        <v>138.9</v>
+      </c>
+      <c r="AX2" t="n">
+        <v>32.15415991749746</v>
+      </c>
+      <c r="AY2" t="n">
         <v>103</v>
       </c>
-      <c r="D2" t="n">
-        <v>163</v>
-      </c>
-      <c r="E2" t="n">
-        <v>118.6</v>
-      </c>
-      <c r="F2" t="n">
-        <v>15.02131818450032</v>
-      </c>
-      <c r="G2" t="n">
-        <v>101</v>
-      </c>
-      <c r="H2" t="n">
-        <v>144</v>
-      </c>
-      <c r="I2" t="n">
-        <v>124.9</v>
-      </c>
-      <c r="J2" t="n">
-        <v>19.10732843701599</v>
-      </c>
-      <c r="K2" t="n">
+      <c r="AZ2" t="n">
+        <v>202</v>
+      </c>
+      <c r="BA2" t="n">
+        <v>111.9</v>
+      </c>
+      <c r="BB2" t="n">
+        <v>19.48050307358616</v>
+      </c>
+      <c r="BC2" t="n">
+        <v>103</v>
+      </c>
+      <c r="BD2" t="n">
+        <v>170</v>
+      </c>
+      <c r="BE2" t="n">
+        <v>111.7</v>
+      </c>
+      <c r="BF2" t="n">
+        <v>17.75415444339718</v>
+      </c>
+      <c r="BG2" t="n">
+        <v>100</v>
+      </c>
+      <c r="BH2" t="n">
+        <v>150</v>
+      </c>
+      <c r="BI2" t="n">
+        <v>110.5</v>
+      </c>
+      <c r="BJ2" t="n">
+        <v>17.74401307483738</v>
+      </c>
+      <c r="BK2" t="n">
+        <v>100</v>
+      </c>
+      <c r="BL2" t="n">
+        <v>154</v>
+      </c>
+      <c r="BM2" t="n">
+        <v>110.6</v>
+      </c>
+      <c r="BN2" t="n">
+        <v>20.96759404414345</v>
+      </c>
+      <c r="BO2" t="n">
+        <v>97</v>
+      </c>
+      <c r="BP2" t="n">
+        <v>173</v>
+      </c>
+      <c r="BQ2" t="n">
+        <v>102.5</v>
+      </c>
+      <c r="BR2" t="n">
+        <v>2.156385865284783</v>
+      </c>
+      <c r="BS2" t="n">
+        <v>100</v>
+      </c>
+      <c r="BT2" t="n">
+        <v>106</v>
+      </c>
+      <c r="BU2" t="n">
+        <v>101.2</v>
+      </c>
+      <c r="BV2" t="n">
+        <v>2.712931993250108</v>
+      </c>
+      <c r="BW2" t="n">
+        <v>98</v>
+      </c>
+      <c r="BX2" t="n">
+        <v>108</v>
+      </c>
+      <c r="BY2" t="n">
+        <v>99.09999999999999</v>
+      </c>
+      <c r="BZ2" t="n">
+        <v>2.343074902771996</v>
+      </c>
+      <c r="CA2" t="n">
+        <v>95</v>
+      </c>
+      <c r="CB2" t="n">
+        <v>102</v>
+      </c>
+      <c r="CC2" t="n">
+        <v>100.3</v>
+      </c>
+      <c r="CD2" t="n">
+        <v>3.195309061734091</v>
+      </c>
+      <c r="CE2" t="n">
+        <v>95</v>
+      </c>
+      <c r="CF2" t="n">
+        <v>106</v>
+      </c>
+      <c r="CG2" t="n">
+        <v>101.4</v>
+      </c>
+      <c r="CH2" t="n">
+        <v>2.2</v>
+      </c>
+      <c r="CI2" t="n">
         <v>99</v>
       </c>
-      <c r="L2" t="n">
-        <v>157</v>
-      </c>
-      <c r="M2" t="n">
-        <v>204</v>
-      </c>
-      <c r="N2" t="n">
-        <v>268.2189404199487</v>
-      </c>
-      <c r="O2" t="n">
-        <v>101</v>
-      </c>
-      <c r="P2" t="n">
-        <v>1008</v>
-      </c>
-      <c r="Q2" t="n">
-        <v>130.4</v>
-      </c>
-      <c r="R2" t="n">
-        <v>50.66201733054064</v>
-      </c>
-      <c r="S2" t="n">
-        <v>101</v>
-      </c>
-      <c r="T2" t="n">
-        <v>271</v>
-      </c>
-      <c r="U2" t="n">
-        <v>400.6</v>
-      </c>
-      <c r="V2" t="n">
-        <v>421.9889098068811</v>
-      </c>
-      <c r="W2" t="n">
+      <c r="CJ2" t="n">
+        <v>106</v>
+      </c>
+      <c r="CK2" t="n">
+        <v>99</v>
+      </c>
+      <c r="CL2" t="n">
+        <v>2.449489742783178</v>
+      </c>
+      <c r="CM2" t="n">
+        <v>95</v>
+      </c>
+      <c r="CN2" t="n">
+        <v>104</v>
+      </c>
+      <c r="CO2" t="n">
+        <v>99.3</v>
+      </c>
+      <c r="CP2" t="n">
+        <v>3.822302970723279</v>
+      </c>
+      <c r="CQ2" t="n">
+        <v>93</v>
+      </c>
+      <c r="CR2" t="n">
+        <v>106</v>
+      </c>
+      <c r="CS2" t="n">
+        <v>96.8</v>
+      </c>
+      <c r="CT2" t="n">
+        <v>3.487119154832539</v>
+      </c>
+      <c r="CU2" t="n">
+        <v>92</v>
+      </c>
+      <c r="CV2" t="n">
         <v>102</v>
       </c>
-      <c r="X2" t="n">
-        <v>1104</v>
-      </c>
-      <c r="Y2" t="n">
-        <v>225.8</v>
-      </c>
-      <c r="Z2" t="n">
-        <v>272.5783557071251</v>
-      </c>
-      <c r="AA2" t="n">
-        <v>100</v>
-      </c>
-      <c r="AB2" t="n">
-        <v>1031</v>
-      </c>
-      <c r="AC2" t="n">
-        <v>107.8</v>
-      </c>
-      <c r="AD2" t="n">
-        <v>20.75957610357205</v>
-      </c>
-      <c r="AE2" t="n">
+      <c r="CW2" t="n">
+        <v>98.09999999999999</v>
+      </c>
+      <c r="CX2" t="n">
+        <v>3.534119409414458</v>
+      </c>
+      <c r="CY2" t="n">
+        <v>93</v>
+      </c>
+      <c r="CZ2" t="n">
+        <v>102</v>
+      </c>
+      <c r="DA2" t="n">
+        <v>99.90000000000001</v>
+      </c>
+      <c r="DB2" t="n">
+        <v>2.808914381037628</v>
+      </c>
+      <c r="DC2" t="n">
+        <v>93</v>
+      </c>
+      <c r="DD2" t="n">
+        <v>103</v>
+      </c>
+      <c r="DE2" t="n">
+        <v>97.59999999999999</v>
+      </c>
+      <c r="DF2" t="n">
+        <v>3.583294573433783</v>
+      </c>
+      <c r="DG2" t="n">
+        <v>92</v>
+      </c>
+      <c r="DH2" t="n">
+        <v>103</v>
+      </c>
+      <c r="DI2" t="n">
+        <v>99.09999999999999</v>
+      </c>
+      <c r="DJ2" t="n">
+        <v>4.570557952810575</v>
+      </c>
+      <c r="DK2" t="n">
+        <v>91</v>
+      </c>
+      <c r="DL2" t="n">
+        <v>107</v>
+      </c>
+      <c r="DM2" t="n">
         <v>99</v>
       </c>
-      <c r="AF2" t="n">
-        <v>170</v>
-      </c>
-      <c r="AG2" t="n">
-        <v>128.3</v>
-      </c>
-      <c r="AH2" t="n">
-        <v>51.9539218923846</v>
-      </c>
-      <c r="AI2" t="n">
-        <v>102</v>
-      </c>
-      <c r="AJ2" t="n">
-        <v>276</v>
-      </c>
-      <c r="AK2" t="n">
-        <v>115.5</v>
-      </c>
-      <c r="AL2" t="n">
-        <v>39.5506005011302</v>
-      </c>
-      <c r="AM2" t="n">
-        <v>100</v>
-      </c>
-      <c r="AN2" t="n">
-        <v>234</v>
-      </c>
-      <c r="AO2" t="n">
-        <v>121.3</v>
-      </c>
-      <c r="AP2" t="n">
-        <v>27.83540910423269</v>
-      </c>
-      <c r="AQ2" t="n">
-        <v>101</v>
-      </c>
-      <c r="AR2" t="n">
-        <v>168</v>
-      </c>
-      <c r="AS2" t="n">
-        <v>130.7</v>
-      </c>
-      <c r="AT2" t="n">
-        <v>40.08752923291731</v>
-      </c>
-      <c r="AU2" t="n">
-        <v>100</v>
-      </c>
-      <c r="AV2" t="n">
-        <v>206</v>
-      </c>
-      <c r="AW2" t="n">
-        <v>120.9</v>
-      </c>
-      <c r="AX2" t="n">
-        <v>28.77307769426135</v>
-      </c>
-      <c r="AY2" t="n">
-        <v>98</v>
-      </c>
-      <c r="AZ2" t="n">
-        <v>176</v>
-      </c>
-      <c r="BA2" t="n">
-        <v>110.1</v>
-      </c>
-      <c r="BB2" t="n">
-        <v>14.51516448408353</v>
-      </c>
-      <c r="BC2" t="n">
-        <v>100</v>
-      </c>
-      <c r="BD2" t="n">
-        <v>148</v>
-      </c>
-      <c r="BE2" t="n">
-        <v>124.5</v>
-      </c>
-      <c r="BF2" t="n">
-        <v>47.81683803849853</v>
-      </c>
-      <c r="BG2" t="n">
-        <v>98</v>
-      </c>
-      <c r="BH2" t="n">
-        <v>261</v>
-      </c>
-      <c r="BI2" t="n">
-        <v>133.8</v>
-      </c>
-      <c r="BJ2" t="n">
-        <v>39.21683312048539</v>
-      </c>
-      <c r="BK2" t="n">
-        <v>97</v>
-      </c>
-      <c r="BL2" t="n">
-        <v>210</v>
-      </c>
-      <c r="BM2" t="n">
-        <v>113.5</v>
-      </c>
-      <c r="BN2" t="n">
-        <v>14.56193668438371</v>
-      </c>
-      <c r="BO2" t="n">
-        <v>103</v>
-      </c>
-      <c r="BP2" t="n">
-        <v>144</v>
-      </c>
-      <c r="BQ2" t="n">
-        <v>125.4</v>
-      </c>
-      <c r="BR2" t="n">
-        <v>49.51807750710845</v>
-      </c>
-      <c r="BS2" t="n">
-        <v>99</v>
-      </c>
-      <c r="BT2" t="n">
-        <v>267</v>
-      </c>
-      <c r="BU2" t="n">
-        <v>113.9</v>
-      </c>
-      <c r="BV2" t="n">
-        <v>26.1283371074395</v>
-      </c>
-      <c r="BW2" t="n">
-        <v>93</v>
-      </c>
-      <c r="BX2" t="n">
-        <v>167</v>
-      </c>
-      <c r="BY2" t="n">
-        <v>170.6</v>
-      </c>
-      <c r="BZ2" t="n">
-        <v>132.3527105880344</v>
-      </c>
-      <c r="CA2" t="n">
-        <v>98</v>
-      </c>
-      <c r="CB2" t="n">
-        <v>560</v>
-      </c>
-      <c r="CC2" t="n">
-        <v>120.3</v>
-      </c>
-      <c r="CD2" t="n">
-        <v>25.06411777821035</v>
-      </c>
-      <c r="CE2" t="n">
-        <v>100</v>
-      </c>
-      <c r="CF2" t="n">
-        <v>171</v>
-      </c>
-      <c r="CG2" t="n">
-        <v>166.7</v>
-      </c>
-      <c r="CH2" t="n">
-        <v>167.4980895413437</v>
-      </c>
-      <c r="CI2" t="n">
-        <v>96</v>
-      </c>
-      <c r="CJ2" t="n">
-        <v>664</v>
-      </c>
-      <c r="CK2" t="n">
-        <v>184.5</v>
-      </c>
-      <c r="CL2" t="n">
-        <v>157.4428467730433</v>
-      </c>
-      <c r="CM2" t="n">
-        <v>98</v>
-      </c>
-      <c r="CN2" t="n">
-        <v>644</v>
-      </c>
-      <c r="CO2" t="n">
-        <v>119</v>
-      </c>
-      <c r="CP2" t="n">
-        <v>22.45439823286298</v>
-      </c>
-      <c r="CQ2" t="n">
-        <v>94</v>
-      </c>
-      <c r="CR2" t="n">
-        <v>165</v>
-      </c>
-      <c r="CS2" t="n">
-        <v>116.1</v>
-      </c>
-      <c r="CT2" t="n">
-        <v>15.4819249449156</v>
-      </c>
-      <c r="CU2" t="n">
-        <v>100</v>
-      </c>
-      <c r="CV2" t="n">
-        <v>140</v>
-      </c>
-      <c r="CW2" t="n">
-        <v>123.1</v>
-      </c>
-      <c r="CX2" t="n">
-        <v>25.02578670092111</v>
-      </c>
-      <c r="CY2" t="n">
-        <v>101</v>
-      </c>
-      <c r="CZ2" t="n">
-        <v>174</v>
-      </c>
-      <c r="DA2" t="n">
-        <v>111.1</v>
-      </c>
-      <c r="DB2" t="n">
-        <v>15.85212919452778</v>
-      </c>
-      <c r="DC2" t="n">
-        <v>99</v>
-      </c>
-      <c r="DD2" t="n">
-        <v>145</v>
-      </c>
-      <c r="DE2" t="n">
-        <v>124</v>
-      </c>
-      <c r="DF2" t="n">
-        <v>20.47437422731156</v>
-      </c>
-      <c r="DG2" t="n">
-        <v>104</v>
-      </c>
-      <c r="DH2" t="n">
-        <v>166</v>
-      </c>
-      <c r="DI2" t="n">
-        <v>114</v>
-      </c>
-      <c r="DJ2" t="n">
-        <v>19.83935482821959</v>
-      </c>
-      <c r="DK2" t="n">
-        <v>98</v>
-      </c>
-      <c r="DL2" t="n">
-        <v>162</v>
-      </c>
-      <c r="DM2" t="n">
-        <v>109.5</v>
-      </c>
       <c r="DN2" t="n">
-        <v>17.68191166135608</v>
+        <v>3.521363372331802</v>
       </c>
       <c r="DO2" t="n">
-        <v>99</v>
+        <v>95</v>
       </c>
       <c r="DP2" t="n">
-        <v>161</v>
+        <v>105</v>
       </c>
       <c r="DQ2" t="n">
-        <v>4233.4</v>
+        <v>7509.599999999999</v>
       </c>
     </row>
   </sheetData>

</xml_diff>